<commit_message>
Audit des limites moteur : 100 tourelles comptées, plafonds à 2 cases du sol
- verifier_limites : bâti ≤ 8 400 structures (y compris au plus fort du
  chantier), exactement 100 tourelles comptées (Heavy + Tek, Tesla hors
  cap), hauteur ≤ 70 murs, aucun plafond à plus de 2 cases d'un appui
  relié au sol ;
- piliers PB du sol à Z2400 (30 plafonds du centre étaient à 3-4 cases) ;
- 4 Tesla de rive sur les côtés E1 et 10 tourelles debout sous le toit
  (5 Tek, 5 Heavy) : 65 H + 35 T + 10 S, le dessus du centre couvert ;
- phases trop grosses coupées en sous-phases (option --appuis prudent) ;
- module 09, docs, matrice et bilan Excel mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WXsGCqXwcUWvE3vyBN5SJi
</commit_message>
<xml_diff>
--- a/donnees/07_bilan_materiaux.xlsx
+++ b/donnees/07_bilan_materiaux.xlsx
@@ -27,7 +27,7 @@
     <t xml:space="preserve">Forteresse Ø30 — bilan matériaux</t>
   </si>
   <si>
-    <t xml:space="preserve">Calculé depuis l'onglet Détail. Les tourelles (60 Heavy, 30 Tek, 6 Tesla) sont déjà en inventaire : ne fabriquez que la colonne « À fabriquer ».</t>
+    <t xml:space="preserve">Calculé depuis l'onglet Détail. Les tourelles (65 Heavy, 35 Tek, 10 Tesla) sont déjà en inventaire : ne fabriquez que la colonne « À fabriquer ».</t>
   </si>
   <si>
     <t xml:space="preserve">Nombre de structures</t>
@@ -195,13 +195,13 @@
     <t xml:space="preserve">Silex</t>
   </si>
   <si>
-    <t xml:space="preserve">Option --appuis prudent (un poteau au bout de chaque ligne de rampes) : +566 piliers fins, soit +7 358 lingots et +2 264 pâte.</t>
+    <t xml:space="preserve">Option --appuis prudent (un poteau au bout de chaque ligne de rampes) : +566 piliers fins, soit +7 358 lingots et +2 264 pâte (145 737 lingots et 36 961 pâte à fabriquer).</t>
   </si>
   <si>
     <t xml:space="preserve">Étoile centrale déjà construite : retirez 87 fondations et 174 triangles (−8 700 lingots, −2 697 pâte) dans l'onglet Détail.</t>
   </si>
   <si>
-    <t xml:space="preserve">Source des quantités : outils/forteresse.py → donnees/synthese.json (bilan_complet), version 92b8c5f.</t>
+    <t xml:space="preserve">Source des quantités : outils/forteresse.py → donnees/synthese.json (bilan_complet). Limites moteur : module 09.</t>
   </si>
   <si>
     <t xml:space="preserve">Bilan matériaux — détail par pièce</t>
@@ -429,7 +429,7 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Le plan 2 contient en plus 36 murs de chaume + 30 Heavy + 6 Tesla, le plan 7 60 murs de chaume + 60 tourelles (onglet Détail).</t>
+    <t xml:space="preserve">Le plan 2 contient en plus 40 murs de chaume + 30 Heavy + 10 Tesla, le plan 6 10 tourelles debout, le plan 7 60 murs de chaume + 60 tourelles (onglet Détail).</t>
   </si>
 </sst>
 </file>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$C$5:$C$29,Détail!$A$5:$A$29,A6)</f>
-        <v>4669</v>
+        <v>4737</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>7</v>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$C$5:$C$29,Détail!$A$5:$A$29,A9)</f>
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>13</v>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$C$5:$C$29,Détail!$A$5:$A$29,A11)</f>
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>17</v>
@@ -1174,11 +1174,11 @@
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">SUM(B6:B11)</f>
-        <v>4989</v>
+        <v>5075</v>
       </c>
       <c r="C12" s="10" t="n">
         <f aca="false">B12-B7-B9</f>
-        <v>4884</v>
+        <v>4966</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -1276,11 +1276,11 @@
       </c>
       <c r="B16" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$R$5:$R$29,Détail!$A$5:$A$29,$A16)</f>
-        <v>108712</v>
+        <v>110412</v>
       </c>
       <c r="C16" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$S$5:$S$29,Détail!$A$5:$A$29,$A16)</f>
-        <v>31285</v>
+        <v>31761</v>
       </c>
       <c r="D16" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$T$5:$T$29,Détail!$A$5:$A$29,$A16)</f>
@@ -1487,15 +1487,15 @@
       </c>
       <c r="L19" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$AB$5:$AB$29,Détail!$A$5:$A$29,$A19)</f>
-        <v>384</v>
+        <v>400</v>
       </c>
       <c r="M19" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$AC$5:$AC$29,Détail!$A$5:$A$29,$A19)</f>
-        <v>672</v>
+        <v>700</v>
       </c>
       <c r="N19" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$AD$5:$AD$29,Détail!$A$5:$A$29,$A19)</f>
-        <v>384</v>
+        <v>400</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1561,27 +1561,27 @@
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$R$5:$R$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>38400</v>
+        <v>43600</v>
       </c>
       <c r="C21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$S$5:$S$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>13500</v>
+        <v>14750</v>
       </c>
       <c r="D21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$T$5:$T$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>19800</v>
+        <v>22050</v>
       </c>
       <c r="E21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$U$5:$U$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>7500</v>
+        <v>9300</v>
       </c>
       <c r="F21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$V$5:$V$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="G21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$W$5:$W$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="H21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$X$5:$X$29,Détail!$A$5:$A$29,$A21)</f>
@@ -1618,11 +1618,11 @@
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">SUM(B16:B20)</f>
-        <v>136679</v>
+        <v>138379</v>
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">SUM(C16:C20)</f>
-        <v>34221</v>
+        <v>34697</v>
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">SUM(D16:D20)</f>
@@ -1658,15 +1658,15 @@
       </c>
       <c r="L22" s="9" t="n">
         <f aca="false">SUM(L16:L20)</f>
-        <v>2604</v>
+        <v>2620</v>
       </c>
       <c r="M22" s="9" t="n">
         <f aca="false">SUM(M16:M20)</f>
-        <v>672</v>
+        <v>700</v>
       </c>
       <c r="N22" s="9" t="n">
         <f aca="false">SUM(N16:N20)</f>
-        <v>384</v>
+        <v>400</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1675,27 +1675,27 @@
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">SUM(B16:B21)</f>
-        <v>175079</v>
+        <v>181979</v>
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">SUM(C16:C21)</f>
-        <v>47721</v>
+        <v>49447</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">SUM(D16:D21)</f>
-        <v>20020</v>
+        <v>22270</v>
       </c>
       <c r="E23" s="9" t="n">
         <f aca="false">SUM(E16:E21)</f>
-        <v>13350</v>
+        <v>15150</v>
       </c>
       <c r="F23" s="9" t="n">
         <f aca="false">SUM(F16:F21)</f>
-        <v>4550</v>
+        <v>5350</v>
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">SUM(G16:G21)</f>
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="H23" s="9" t="n">
         <f aca="false">SUM(H16:H21)</f>
@@ -1715,15 +1715,15 @@
       </c>
       <c r="L23" s="9" t="n">
         <f aca="false">SUM(L16:L21)</f>
-        <v>2604</v>
+        <v>2620</v>
       </c>
       <c r="M23" s="9" t="n">
         <f aca="false">SUM(M16:M21)</f>
-        <v>672</v>
+        <v>700</v>
       </c>
       <c r="N23" s="9" t="n">
         <f aca="false">SUM(N16:N21)</f>
-        <v>384</v>
+        <v>400</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2002,11 +2002,11 @@
       </c>
       <c r="B38" s="14" t="n">
         <f aca="false">(B22+$B$29*D22)</f>
-        <v>136899</v>
+        <v>138599</v>
       </c>
       <c r="C38" s="14" t="n">
         <f aca="false">(B23+$B$29*D23)</f>
-        <v>195099</v>
+        <v>204249</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
@@ -2026,11 +2026,11 @@
       </c>
       <c r="B39" s="14" t="n">
         <f aca="false">$B$27*(B22+$B$29*D22)</f>
-        <v>273798</v>
+        <v>277198</v>
       </c>
       <c r="C39" s="14" t="n">
         <f aca="false">$B$27*(B23+$B$29*D23)</f>
-        <v>390198</v>
+        <v>408498</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -2050,11 +2050,11 @@
       </c>
       <c r="B40" s="14" t="n">
         <f aca="false">(C22+$B$31*E22)</f>
-        <v>45921</v>
+        <v>46397</v>
       </c>
       <c r="C40" s="14" t="n">
         <f aca="false">(C23+$B$31*E23)</f>
-        <v>74421</v>
+        <v>79747</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
@@ -2074,11 +2074,11 @@
       </c>
       <c r="B41" s="14" t="n">
         <f aca="false">$B$32*(C22+$B$31*E22)</f>
-        <v>183684</v>
+        <v>185588</v>
       </c>
       <c r="C41" s="14" t="n">
         <f aca="false">$B$32*(C23+$B$31*E23)</f>
-        <v>297684</v>
+        <v>318988</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -2098,11 +2098,11 @@
       </c>
       <c r="B42" s="14" t="n">
         <f aca="false">$B$33*(C22+$B$31*E22)+$B$35*J22</f>
-        <v>367468</v>
+        <v>371276</v>
       </c>
       <c r="C42" s="14" t="n">
         <f aca="false">$B$33*(C23+$B$31*E23)+$B$35*J23</f>
-        <v>595468</v>
+        <v>638076</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="C43" s="14" t="n">
         <f aca="false">$B$30*E23</f>
-        <v>26700</v>
+        <v>30300</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="C44" s="14" t="n">
         <f aca="false">$B$28*D23</f>
-        <v>60060</v>
+        <v>66810</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
@@ -2484,7 +2484,7 @@
         <v>91</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1076</v>
+        <v>1072</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="16" t="n">
@@ -2528,11 +2528,11 @@
       </c>
       <c r="R5" s="14" t="n">
         <f aca="false">$C5*E5</f>
-        <v>26900</v>
+        <v>26800</v>
       </c>
       <c r="S5" s="14" t="n">
         <f aca="false">$C5*F5</f>
-        <v>7532</v>
+        <v>7504</v>
       </c>
       <c r="T5" s="14" t="n">
         <f aca="false">$C5*G5</f>
@@ -2900,7 +2900,7 @@
         <v>96</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>346</v>
+        <v>418</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="16" t="n">
@@ -2944,11 +2944,11 @@
       </c>
       <c r="R9" s="14" t="n">
         <f aca="false">$C9*E9</f>
-        <v>8650</v>
+        <v>10450</v>
       </c>
       <c r="S9" s="14" t="n">
         <f aca="false">$C9*F9</f>
-        <v>2422</v>
+        <v>2926</v>
       </c>
       <c r="T9" s="14" t="n">
         <f aca="false">$C9*G9</f>
@@ -4047,7 +4047,7 @@
         <v>107</v>
       </c>
       <c r="C20" s="15" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>93</v>
@@ -4133,15 +4133,15 @@
       </c>
       <c r="AB20" s="14" t="n">
         <f aca="false">$C20*O20</f>
-        <v>384</v>
+        <v>400</v>
       </c>
       <c r="AC20" s="14" t="n">
         <f aca="false">$C20*P20</f>
-        <v>672</v>
+        <v>700</v>
       </c>
       <c r="AD20" s="14" t="n">
         <f aca="false">$C20*Q20</f>
-        <v>384</v>
+        <v>400</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4772,7 +4772,7 @@
         <v>114</v>
       </c>
       <c r="C27" s="15" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="16" t="n">
@@ -4816,19 +4816,19 @@
       </c>
       <c r="R27" s="14" t="n">
         <f aca="false">$C27*E27</f>
-        <v>32400</v>
+        <v>35100</v>
       </c>
       <c r="S27" s="14" t="n">
         <f aca="false">$C27*F27</f>
-        <v>12000</v>
+        <v>13000</v>
       </c>
       <c r="T27" s="14" t="n">
         <f aca="false">$C27*G27</f>
-        <v>16200</v>
+        <v>17550</v>
       </c>
       <c r="U27" s="14" t="n">
         <f aca="false">$C27*H27</f>
-        <v>4200</v>
+        <v>4550</v>
       </c>
       <c r="V27" s="14" t="n">
         <f aca="false">$C27*I27</f>
@@ -4875,7 +4875,7 @@
         <v>115</v>
       </c>
       <c r="C28" s="15" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="16" t="n">
@@ -4919,19 +4919,19 @@
       </c>
       <c r="R28" s="14" t="n">
         <f aca="false">$C28*E28</f>
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="S28" s="14" t="n">
         <f aca="false">$C28*F28</f>
-        <v>1500</v>
+        <v>1750</v>
       </c>
       <c r="T28" s="14" t="n">
         <f aca="false">$C28*G28</f>
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="U28" s="14" t="n">
         <f aca="false">$C28*H28</f>
-        <v>1500</v>
+        <v>1750</v>
       </c>
       <c r="V28" s="14" t="n">
         <f aca="false">$C28*I28</f>
@@ -4939,7 +4939,7 @@
       </c>
       <c r="W28" s="14" t="n">
         <f aca="false">$C28*J28</f>
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="X28" s="14" t="n">
         <f aca="false">$C28*K28</f>
@@ -4978,7 +4978,7 @@
         <v>116</v>
       </c>
       <c r="C29" s="15" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="16" t="n">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="R29" s="14" t="n">
         <f aca="false">$C29*E29</f>
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="S29" s="14" t="n">
         <f aca="false">$C29*F29</f>
@@ -5030,15 +5030,15 @@
       </c>
       <c r="T29" s="14" t="n">
         <f aca="false">$C29*G29</f>
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="U29" s="14" t="n">
         <f aca="false">$C29*H29</f>
-        <v>1800</v>
+        <v>3000</v>
       </c>
       <c r="V29" s="14" t="n">
         <f aca="false">$C29*I29</f>
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="W29" s="14" t="n">
         <f aca="false">$C29*J29</f>
@@ -5080,7 +5080,7 @@
       <c r="B30" s="17"/>
       <c r="C30" s="8" t="n">
         <f aca="false">SUM(C5:C29)</f>
-        <v>4989</v>
+        <v>5075</v>
       </c>
       <c r="D30" s="17"/>
       <c r="E30" s="17"/>
@@ -5098,27 +5098,27 @@
       <c r="Q30" s="17"/>
       <c r="R30" s="9" t="n">
         <f aca="false">SUM(R5:R29)</f>
-        <v>175079</v>
+        <v>181979</v>
       </c>
       <c r="S30" s="9" t="n">
         <f aca="false">SUM(S5:S29)</f>
-        <v>47721</v>
+        <v>49447</v>
       </c>
       <c r="T30" s="9" t="n">
         <f aca="false">SUM(T5:T29)</f>
-        <v>20020</v>
+        <v>22270</v>
       </c>
       <c r="U30" s="9" t="n">
         <f aca="false">SUM(U5:U29)</f>
-        <v>13350</v>
+        <v>15150</v>
       </c>
       <c r="V30" s="9" t="n">
         <f aca="false">SUM(V5:V29)</f>
-        <v>4550</v>
+        <v>5350</v>
       </c>
       <c r="W30" s="9" t="n">
         <f aca="false">SUM(W5:W29)</f>
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="X30" s="9" t="n">
         <f aca="false">SUM(X5:X29)</f>
@@ -5138,15 +5138,15 @@
       </c>
       <c r="AB30" s="9" t="n">
         <f aca="false">SUM(AB5:AB29)</f>
-        <v>2604</v>
+        <v>2620</v>
       </c>
       <c r="AC30" s="9" t="n">
         <f aca="false">SUM(AC5:AC29)</f>
-        <v>672</v>
+        <v>700</v>
       </c>
       <c r="AD30" s="9" t="n">
         <f aca="false">SUM(AD5:AD29)</f>
-        <v>384</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -5467,7 +5467,7 @@
         <v>127</v>
       </c>
       <c r="B8" s="16" t="n">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>564</v>
@@ -5507,15 +5507,15 @@
       </c>
       <c r="O8" s="20" t="n">
         <f aca="false">SUM(B8:N8)</f>
-        <v>1369</v>
+        <v>1365</v>
       </c>
       <c r="P8" s="20" t="n">
         <f aca="false">SUMPRODUCT(B8:N8,B$4:N$4)</f>
-        <v>23515</v>
+        <v>23415</v>
       </c>
       <c r="Q8" s="20" t="n">
         <f aca="false">SUMPRODUCT(B8:N8,B$5:N$5)</f>
-        <v>6461</v>
+        <v>6433</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5591,7 +5591,7 @@
         <v>170</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>120</v>
+        <v>192</v>
       </c>
       <c r="G10" s="16" t="n">
         <v>0</v>
@@ -5619,15 +5619,15 @@
       </c>
       <c r="O10" s="20" t="n">
         <f aca="false">SUM(B10:N10)</f>
-        <v>794</v>
+        <v>866</v>
       </c>
       <c r="P10" s="20" t="n">
         <f aca="false">SUMPRODUCT(B10:N10,B$4:N$4)</f>
-        <v>19660</v>
+        <v>21460</v>
       </c>
       <c r="Q10" s="20" t="n">
         <f aca="false">SUMPRODUCT(B10:N10,B$5:N$5)</f>
-        <v>5521</v>
+        <v>6025</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5860,7 +5860,7 @@
       </c>
       <c r="B15" s="21" t="n">
         <f aca="false">SUM(B7:B14)</f>
-        <v>1076</v>
+        <v>1072</v>
       </c>
       <c r="C15" s="21" t="n">
         <f aca="false">SUM(C7:C14)</f>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="F15" s="21" t="n">
         <f aca="false">SUM(F7:F14)</f>
-        <v>346</v>
+        <v>418</v>
       </c>
       <c r="G15" s="21" t="n">
         <f aca="false">SUM(G7:G14)</f>
@@ -5912,15 +5912,15 @@
       </c>
       <c r="O15" s="21" t="n">
         <f aca="false">SUM(O7:O14)</f>
-        <v>4669</v>
+        <v>4737</v>
       </c>
       <c r="P15" s="21" t="n">
         <f aca="false">SUM(P7:P14)</f>
-        <v>108712</v>
+        <v>110412</v>
       </c>
       <c r="Q15" s="21" t="n">
         <f aca="false">SUM(Q7:Q14)</f>
-        <v>31285</v>
+        <v>31761</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Tesla comptées dans le cap : 100 tourelles (62 Heavy, 32 Tek, 6 Tesla)
Les Tesla comptent sur le serveur : tesla_comptee=True. Les 4 Tesla de rive
des côtés E1 sont retirées (la rive retrouve ses 143 murs) et le toit garde
4 tourelles debout (2 Tek, 2 Heavy) au lieu de 10, pour un cap plein à 100
avec L1 complet. Piliers PB toujours du sol au toit. Module 09, docs,
matrice et bilan Excel mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WXsGCqXwcUWvE3vyBN5SJi
</commit_message>
<xml_diff>
--- a/donnees/07_bilan_materiaux.xlsx
+++ b/donnees/07_bilan_materiaux.xlsx
@@ -27,7 +27,7 @@
     <t xml:space="preserve">Forteresse Ø30 — bilan matériaux</t>
   </si>
   <si>
-    <t xml:space="preserve">Calculé depuis l'onglet Détail. Les tourelles (65 Heavy, 35 Tek, 10 Tesla) sont déjà en inventaire : ne fabriquez que la colonne « À fabriquer ».</t>
+    <t xml:space="preserve">Calculé depuis l'onglet Détail. Les tourelles (62 Heavy, 32 Tek, 6 Tesla) sont déjà en inventaire : ne fabriquez que la colonne « À fabriquer ».</t>
   </si>
   <si>
     <t xml:space="preserve">Nombre de structures</t>
@@ -195,7 +195,7 @@
     <t xml:space="preserve">Silex</t>
   </si>
   <si>
-    <t xml:space="preserve">Option --appuis prudent (un poteau au bout de chaque ligne de rampes) : +566 piliers fins, soit +7 358 lingots et +2 264 pâte (145 737 lingots et 36 961 pâte à fabriquer).</t>
+    <t xml:space="preserve">Option --appuis prudent (un poteau au bout de chaque ligne de rampes) : +566 piliers fins, soit +7 358 lingots et +2 264 pâte (145 837 lingots et 36 989 pâte à fabriquer).</t>
   </si>
   <si>
     <t xml:space="preserve">Étoile centrale déjà construite : retirez 87 fondations et 174 triangles (−8 700 lingots, −2 697 pâte) dans l'onglet Détail.</t>
@@ -429,7 +429,7 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Le plan 2 contient en plus 40 murs de chaume + 30 Heavy + 10 Tesla, le plan 6 10 tourelles debout, le plan 7 60 murs de chaume + 60 tourelles (onglet Détail).</t>
+    <t xml:space="preserve">Le plan 2 contient en plus 36 murs de chaume + 30 Heavy + 6 Tesla, le plan 6 4 tourelles debout, le plan 7 60 murs de chaume + 60 tourelles (onglet Détail).</t>
   </si>
 </sst>
 </file>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$C$5:$C$29,Détail!$A$5:$A$29,A6)</f>
-        <v>4737</v>
+        <v>4741</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>7</v>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$C$5:$C$29,Détail!$A$5:$A$29,A9)</f>
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>13</v>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$C$5:$C$29,Détail!$A$5:$A$29,A11)</f>
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>17</v>
@@ -1174,11 +1174,11 @@
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">SUM(B6:B11)</f>
-        <v>5075</v>
+        <v>5065</v>
       </c>
       <c r="C12" s="10" t="n">
         <f aca="false">B12-B7-B9</f>
-        <v>4966</v>
+        <v>4960</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -1276,11 +1276,11 @@
       </c>
       <c r="B16" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$R$5:$R$29,Détail!$A$5:$A$29,$A16)</f>
-        <v>110412</v>
+        <v>110512</v>
       </c>
       <c r="C16" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$S$5:$S$29,Détail!$A$5:$A$29,$A16)</f>
-        <v>31761</v>
+        <v>31789</v>
       </c>
       <c r="D16" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$T$5:$T$29,Détail!$A$5:$A$29,$A16)</f>
@@ -1487,15 +1487,15 @@
       </c>
       <c r="L19" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$AB$5:$AB$29,Détail!$A$5:$A$29,$A19)</f>
-        <v>400</v>
+        <v>384</v>
       </c>
       <c r="M19" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$AC$5:$AC$29,Détail!$A$5:$A$29,$A19)</f>
-        <v>700</v>
+        <v>672</v>
       </c>
       <c r="N19" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$AD$5:$AD$29,Détail!$A$5:$A$29,$A19)</f>
-        <v>400</v>
+        <v>384</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1561,27 +1561,27 @@
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$R$5:$R$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>43600</v>
+        <v>39680</v>
       </c>
       <c r="C21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$S$5:$S$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>14750</v>
+        <v>14000</v>
       </c>
       <c r="D21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$T$5:$T$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>22050</v>
+        <v>20540</v>
       </c>
       <c r="E21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$U$5:$U$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>9300</v>
+        <v>7740</v>
       </c>
       <c r="F21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$V$5:$V$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="G21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$W$5:$W$29,Détail!$A$5:$A$29,$A21)</f>
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="H21" s="7" t="n">
         <f aca="false">SUMIFS(Détail!$X$5:$X$29,Détail!$A$5:$A$29,$A21)</f>
@@ -1618,11 +1618,11 @@
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">SUM(B16:B20)</f>
-        <v>138379</v>
+        <v>138479</v>
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">SUM(C16:C20)</f>
-        <v>34697</v>
+        <v>34725</v>
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">SUM(D16:D20)</f>
@@ -1658,15 +1658,15 @@
       </c>
       <c r="L22" s="9" t="n">
         <f aca="false">SUM(L16:L20)</f>
-        <v>2620</v>
+        <v>2604</v>
       </c>
       <c r="M22" s="9" t="n">
         <f aca="false">SUM(M16:M20)</f>
-        <v>700</v>
+        <v>672</v>
       </c>
       <c r="N22" s="9" t="n">
         <f aca="false">SUM(N16:N20)</f>
-        <v>400</v>
+        <v>384</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1675,27 +1675,27 @@
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">SUM(B16:B21)</f>
-        <v>181979</v>
+        <v>178159</v>
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">SUM(C16:C21)</f>
-        <v>49447</v>
+        <v>48725</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">SUM(D16:D21)</f>
-        <v>22270</v>
+        <v>20760</v>
       </c>
       <c r="E23" s="9" t="n">
         <f aca="false">SUM(E16:E21)</f>
-        <v>15150</v>
+        <v>13590</v>
       </c>
       <c r="F23" s="9" t="n">
         <f aca="false">SUM(F16:F21)</f>
-        <v>5350</v>
+        <v>4550</v>
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">SUM(G16:G21)</f>
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="H23" s="9" t="n">
         <f aca="false">SUM(H16:H21)</f>
@@ -1715,15 +1715,15 @@
       </c>
       <c r="L23" s="9" t="n">
         <f aca="false">SUM(L16:L21)</f>
-        <v>2620</v>
+        <v>2604</v>
       </c>
       <c r="M23" s="9" t="n">
         <f aca="false">SUM(M16:M21)</f>
-        <v>700</v>
+        <v>672</v>
       </c>
       <c r="N23" s="9" t="n">
         <f aca="false">SUM(N16:N21)</f>
-        <v>400</v>
+        <v>384</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2002,11 +2002,11 @@
       </c>
       <c r="B38" s="14" t="n">
         <f aca="false">(B22+$B$29*D22)</f>
-        <v>138599</v>
+        <v>138699</v>
       </c>
       <c r="C38" s="14" t="n">
         <f aca="false">(B23+$B$29*D23)</f>
-        <v>204249</v>
+        <v>198919</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
@@ -2026,11 +2026,11 @@
       </c>
       <c r="B39" s="14" t="n">
         <f aca="false">$B$27*(B22+$B$29*D22)</f>
-        <v>277198</v>
+        <v>277398</v>
       </c>
       <c r="C39" s="14" t="n">
         <f aca="false">$B$27*(B23+$B$29*D23)</f>
-        <v>408498</v>
+        <v>397838</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -2050,11 +2050,11 @@
       </c>
       <c r="B40" s="14" t="n">
         <f aca="false">(C22+$B$31*E22)</f>
-        <v>46397</v>
+        <v>46425</v>
       </c>
       <c r="C40" s="14" t="n">
         <f aca="false">(C23+$B$31*E23)</f>
-        <v>79747</v>
+        <v>75905</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
@@ -2074,11 +2074,11 @@
       </c>
       <c r="B41" s="14" t="n">
         <f aca="false">$B$32*(C22+$B$31*E22)</f>
-        <v>185588</v>
+        <v>185700</v>
       </c>
       <c r="C41" s="14" t="n">
         <f aca="false">$B$32*(C23+$B$31*E23)</f>
-        <v>318988</v>
+        <v>303620</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -2098,11 +2098,11 @@
       </c>
       <c r="B42" s="14" t="n">
         <f aca="false">$B$33*(C22+$B$31*E22)+$B$35*J22</f>
-        <v>371276</v>
+        <v>371500</v>
       </c>
       <c r="C42" s="14" t="n">
         <f aca="false">$B$33*(C23+$B$31*E23)+$B$35*J23</f>
-        <v>638076</v>
+        <v>607340</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="C43" s="14" t="n">
         <f aca="false">$B$30*E23</f>
-        <v>30300</v>
+        <v>27180</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="C44" s="14" t="n">
         <f aca="false">$B$28*D23</f>
-        <v>66810</v>
+        <v>62280</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
@@ -2484,7 +2484,7 @@
         <v>91</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1072</v>
+        <v>1076</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="16" t="n">
@@ -2528,11 +2528,11 @@
       </c>
       <c r="R5" s="14" t="n">
         <f aca="false">$C5*E5</f>
-        <v>26800</v>
+        <v>26900</v>
       </c>
       <c r="S5" s="14" t="n">
         <f aca="false">$C5*F5</f>
-        <v>7504</v>
+        <v>7532</v>
       </c>
       <c r="T5" s="14" t="n">
         <f aca="false">$C5*G5</f>
@@ -4047,7 +4047,7 @@
         <v>107</v>
       </c>
       <c r="C20" s="15" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>93</v>
@@ -4133,15 +4133,15 @@
       </c>
       <c r="AB20" s="14" t="n">
         <f aca="false">$C20*O20</f>
-        <v>400</v>
+        <v>384</v>
       </c>
       <c r="AC20" s="14" t="n">
         <f aca="false">$C20*P20</f>
-        <v>700</v>
+        <v>672</v>
       </c>
       <c r="AD20" s="14" t="n">
         <f aca="false">$C20*Q20</f>
-        <v>400</v>
+        <v>384</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4772,7 +4772,7 @@
         <v>114</v>
       </c>
       <c r="C27" s="15" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="16" t="n">
@@ -4816,19 +4816,19 @@
       </c>
       <c r="R27" s="14" t="n">
         <f aca="false">$C27*E27</f>
-        <v>35100</v>
+        <v>33480</v>
       </c>
       <c r="S27" s="14" t="n">
         <f aca="false">$C27*F27</f>
-        <v>13000</v>
+        <v>12400</v>
       </c>
       <c r="T27" s="14" t="n">
         <f aca="false">$C27*G27</f>
-        <v>17550</v>
+        <v>16740</v>
       </c>
       <c r="U27" s="14" t="n">
         <f aca="false">$C27*H27</f>
-        <v>4550</v>
+        <v>4340</v>
       </c>
       <c r="V27" s="14" t="n">
         <f aca="false">$C27*I27</f>
@@ -4875,7 +4875,7 @@
         <v>115</v>
       </c>
       <c r="C28" s="15" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="16" t="n">
@@ -4919,19 +4919,19 @@
       </c>
       <c r="R28" s="14" t="n">
         <f aca="false">$C28*E28</f>
-        <v>3500</v>
+        <v>3200</v>
       </c>
       <c r="S28" s="14" t="n">
         <f aca="false">$C28*F28</f>
-        <v>1750</v>
+        <v>1600</v>
       </c>
       <c r="T28" s="14" t="n">
         <f aca="false">$C28*G28</f>
-        <v>3500</v>
+        <v>3200</v>
       </c>
       <c r="U28" s="14" t="n">
         <f aca="false">$C28*H28</f>
-        <v>1750</v>
+        <v>1600</v>
       </c>
       <c r="V28" s="14" t="n">
         <f aca="false">$C28*I28</f>
@@ -4939,7 +4939,7 @@
       </c>
       <c r="W28" s="14" t="n">
         <f aca="false">$C28*J28</f>
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="X28" s="14" t="n">
         <f aca="false">$C28*K28</f>
@@ -4978,7 +4978,7 @@
         <v>116</v>
       </c>
       <c r="C29" s="15" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="16" t="n">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="R29" s="14" t="n">
         <f aca="false">$C29*E29</f>
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="S29" s="14" t="n">
         <f aca="false">$C29*F29</f>
@@ -5030,15 +5030,15 @@
       </c>
       <c r="T29" s="14" t="n">
         <f aca="false">$C29*G29</f>
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="U29" s="14" t="n">
         <f aca="false">$C29*H29</f>
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="V29" s="14" t="n">
         <f aca="false">$C29*I29</f>
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="W29" s="14" t="n">
         <f aca="false">$C29*J29</f>
@@ -5080,7 +5080,7 @@
       <c r="B30" s="17"/>
       <c r="C30" s="8" t="n">
         <f aca="false">SUM(C5:C29)</f>
-        <v>5075</v>
+        <v>5065</v>
       </c>
       <c r="D30" s="17"/>
       <c r="E30" s="17"/>
@@ -5098,27 +5098,27 @@
       <c r="Q30" s="17"/>
       <c r="R30" s="9" t="n">
         <f aca="false">SUM(R5:R29)</f>
-        <v>181979</v>
+        <v>178159</v>
       </c>
       <c r="S30" s="9" t="n">
         <f aca="false">SUM(S5:S29)</f>
-        <v>49447</v>
+        <v>48725</v>
       </c>
       <c r="T30" s="9" t="n">
         <f aca="false">SUM(T5:T29)</f>
-        <v>22270</v>
+        <v>20760</v>
       </c>
       <c r="U30" s="9" t="n">
         <f aca="false">SUM(U5:U29)</f>
-        <v>15150</v>
+        <v>13590</v>
       </c>
       <c r="V30" s="9" t="n">
         <f aca="false">SUM(V5:V29)</f>
-        <v>5350</v>
+        <v>4550</v>
       </c>
       <c r="W30" s="9" t="n">
         <f aca="false">SUM(W5:W29)</f>
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="X30" s="9" t="n">
         <f aca="false">SUM(X5:X29)</f>
@@ -5138,15 +5138,15 @@
       </c>
       <c r="AB30" s="9" t="n">
         <f aca="false">SUM(AB5:AB29)</f>
-        <v>2620</v>
+        <v>2604</v>
       </c>
       <c r="AC30" s="9" t="n">
         <f aca="false">SUM(AC5:AC29)</f>
-        <v>700</v>
+        <v>672</v>
       </c>
       <c r="AD30" s="9" t="n">
         <f aca="false">SUM(AD5:AD29)</f>
-        <v>400</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -5467,7 +5467,7 @@
         <v>127</v>
       </c>
       <c r="B8" s="16" t="n">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>564</v>
@@ -5507,15 +5507,15 @@
       </c>
       <c r="O8" s="20" t="n">
         <f aca="false">SUM(B8:N8)</f>
-        <v>1365</v>
+        <v>1369</v>
       </c>
       <c r="P8" s="20" t="n">
         <f aca="false">SUMPRODUCT(B8:N8,B$4:N$4)</f>
-        <v>23415</v>
+        <v>23515</v>
       </c>
       <c r="Q8" s="20" t="n">
         <f aca="false">SUMPRODUCT(B8:N8,B$5:N$5)</f>
-        <v>6433</v>
+        <v>6461</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5860,7 +5860,7 @@
       </c>
       <c r="B15" s="21" t="n">
         <f aca="false">SUM(B7:B14)</f>
-        <v>1072</v>
+        <v>1076</v>
       </c>
       <c r="C15" s="21" t="n">
         <f aca="false">SUM(C7:C14)</f>
@@ -5912,15 +5912,15 @@
       </c>
       <c r="O15" s="21" t="n">
         <f aca="false">SUM(O7:O14)</f>
-        <v>4737</v>
+        <v>4741</v>
       </c>
       <c r="P15" s="21" t="n">
         <f aca="false">SUM(P7:P14)</f>
-        <v>110412</v>
+        <v>110512</v>
       </c>
       <c r="Q15" s="21" t="n">
         <f aca="false">SUM(Q7:Q14)</f>
-        <v>31761</v>
+        <v>31789</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>